<commit_message>
Remove obsolete orders from Clean_Ecommerce.csv and update related files
</commit_message>
<xml_diff>
--- a/Clean_Ecommerce.xlsx
+++ b/Clean_Ecommerce.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U381"/>
+  <dimension ref="A1:U371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31839,846 +31839,6 @@
         </is>
       </c>
     </row>
-    <row r="372">
-      <c r="A372" t="inlineStr">
-        <is>
-          <t>ORD1600</t>
-        </is>
-      </c>
-      <c r="B372" s="2" t="n">
-        <v>45792</v>
-      </c>
-      <c r="C372" t="inlineStr">
-        <is>
-          <t>Priya</t>
-        </is>
-      </c>
-      <c r="D372" t="inlineStr">
-        <is>
-          <t>priya67@gmail.com</t>
-        </is>
-      </c>
-      <c r="E372" t="n">
-        <v>9848200695</v>
-      </c>
-      <c r="F372" t="inlineStr">
-        <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="G372" t="inlineStr">
-        <is>
-          <t>Maharashtra</t>
-        </is>
-      </c>
-      <c r="H372" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="I372" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="J372" t="n">
-        <v>3</v>
-      </c>
-      <c r="K372" t="inlineStr"/>
-      <c r="L372" t="n">
-        <v>15</v>
-      </c>
-      <c r="M372" t="inlineStr">
-        <is>
-          <t>UPI</t>
-        </is>
-      </c>
-      <c r="N372" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
-      <c r="O372" s="2" t="n">
-        <v>45792</v>
-      </c>
-      <c r="P372" t="inlineStr"/>
-      <c r="Q372" t="inlineStr"/>
-      <c r="R372" t="inlineStr"/>
-      <c r="S372" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="T372" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U372" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" t="inlineStr">
-        <is>
-          <t>ORD1602</t>
-        </is>
-      </c>
-      <c r="B373" s="2" t="n">
-        <v>45838</v>
-      </c>
-      <c r="C373" t="inlineStr">
-        <is>
-          <t>Neha</t>
-        </is>
-      </c>
-      <c r="D373" t="inlineStr">
-        <is>
-          <t>neha82@gmail.com</t>
-        </is>
-      </c>
-      <c r="E373" t="n">
-        <v>9829008196</v>
-      </c>
-      <c r="F373" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="G373" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="H373" t="inlineStr">
-        <is>
-          <t>Chair</t>
-        </is>
-      </c>
-      <c r="I373" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="J373" t="n">
-        <v>4</v>
-      </c>
-      <c r="K373" t="n">
-        <v>1999</v>
-      </c>
-      <c r="L373" t="n">
-        <v>0</v>
-      </c>
-      <c r="M373" t="inlineStr">
-        <is>
-          <t>UPI</t>
-        </is>
-      </c>
-      <c r="N373" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="O373" s="2" t="n">
-        <v>45723</v>
-      </c>
-      <c r="P373" t="n">
-        <v>7996</v>
-      </c>
-      <c r="Q373" t="n">
-        <v>7996</v>
-      </c>
-      <c r="R373" t="n">
-        <v>1599.2</v>
-      </c>
-      <c r="S373" t="inlineStr">
-        <is>
-          <t>June</t>
-        </is>
-      </c>
-      <c r="T373" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U373" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" t="inlineStr">
-        <is>
-          <t>ORD1603</t>
-        </is>
-      </c>
-      <c r="B374" s="2" t="n">
-        <v>45691</v>
-      </c>
-      <c r="C374" t="inlineStr">
-        <is>
-          <t>Rohit</t>
-        </is>
-      </c>
-      <c r="D374" t="inlineStr">
-        <is>
-          <t>rohit45@gmail.com</t>
-        </is>
-      </c>
-      <c r="E374" t="n">
-        <v>9280491167</v>
-      </c>
-      <c r="F374" t="inlineStr">
-        <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="G374" t="inlineStr">
-        <is>
-          <t>Maharashtra</t>
-        </is>
-      </c>
-      <c r="H374" t="inlineStr">
-        <is>
-          <t>Watch</t>
-        </is>
-      </c>
-      <c r="I374" t="inlineStr">
-        <is>
-          <t>Fashion</t>
-        </is>
-      </c>
-      <c r="J374" t="n">
-        <v>5</v>
-      </c>
-      <c r="K374" t="n">
-        <v>4999</v>
-      </c>
-      <c r="L374" t="n">
-        <v>20</v>
-      </c>
-      <c r="M374" t="inlineStr">
-        <is>
-          <t>Card</t>
-        </is>
-      </c>
-      <c r="N374" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="O374" s="2" t="n">
-        <v>45902</v>
-      </c>
-      <c r="P374" t="n">
-        <v>24995</v>
-      </c>
-      <c r="Q374" t="n">
-        <v>19996</v>
-      </c>
-      <c r="R374" t="n">
-        <v>3999.2</v>
-      </c>
-      <c r="S374" t="inlineStr">
-        <is>
-          <t>February</t>
-        </is>
-      </c>
-      <c r="T374" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U374" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-    </row>
-    <row r="375">
-      <c r="A375" t="inlineStr">
-        <is>
-          <t>ORD1604</t>
-        </is>
-      </c>
-      <c r="B375" s="2" t="n">
-        <v>45783</v>
-      </c>
-      <c r="C375" t="inlineStr">
-        <is>
-          <t>Amit</t>
-        </is>
-      </c>
-      <c r="D375" t="inlineStr">
-        <is>
-          <t>amit6@gmail.com</t>
-        </is>
-      </c>
-      <c r="E375" t="n">
-        <v>9943310925</v>
-      </c>
-      <c r="F375" t="inlineStr">
-        <is>
-          <t>Jaipur</t>
-        </is>
-      </c>
-      <c r="G375" t="inlineStr">
-        <is>
-          <t>Rajasthan</t>
-        </is>
-      </c>
-      <c r="H375" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="I375" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="J375" t="n">
-        <v>3</v>
-      </c>
-      <c r="K375" t="n">
-        <v>1999</v>
-      </c>
-      <c r="L375" t="n">
-        <v>5</v>
-      </c>
-      <c r="M375" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="N375" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="O375" s="2" t="n">
-        <v>45874</v>
-      </c>
-      <c r="P375" t="n">
-        <v>5997</v>
-      </c>
-      <c r="Q375" t="n">
-        <v>5697.15</v>
-      </c>
-      <c r="R375" t="n">
-        <v>1139.43</v>
-      </c>
-      <c r="S375" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="T375" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U375" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-    </row>
-    <row r="376">
-      <c r="A376" t="inlineStr">
-        <is>
-          <t>ORD1607</t>
-        </is>
-      </c>
-      <c r="B376" s="2" t="n">
-        <v>45698</v>
-      </c>
-      <c r="C376" t="inlineStr">
-        <is>
-          <t>Rahul</t>
-        </is>
-      </c>
-      <c r="D376" t="inlineStr">
-        <is>
-          <t>rahul82@gmail.com</t>
-        </is>
-      </c>
-      <c r="E376" t="n">
-        <v>9517780193</v>
-      </c>
-      <c r="F376" t="inlineStr">
-        <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="G376" t="inlineStr">
-        <is>
-          <t>Maharashtra</t>
-        </is>
-      </c>
-      <c r="H376" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="I376" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="J376" t="n">
-        <v>3</v>
-      </c>
-      <c r="K376" t="n">
-        <v>499</v>
-      </c>
-      <c r="L376" t="n">
-        <v>20</v>
-      </c>
-      <c r="M376" t="inlineStr">
-        <is>
-          <t>Wallet</t>
-        </is>
-      </c>
-      <c r="N376" t="inlineStr">
-        <is>
-          <t>Cancelled</t>
-        </is>
-      </c>
-      <c r="O376" s="2" t="n">
-        <v>45698</v>
-      </c>
-      <c r="P376" t="n">
-        <v>1497</v>
-      </c>
-      <c r="Q376" t="n">
-        <v>1197.6</v>
-      </c>
-      <c r="R376" t="n">
-        <v>239.52</v>
-      </c>
-      <c r="S376" t="inlineStr">
-        <is>
-          <t>February</t>
-        </is>
-      </c>
-      <c r="T376" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U376" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" t="inlineStr">
-        <is>
-          <t>ORD1608</t>
-        </is>
-      </c>
-      <c r="B377" s="2" t="n">
-        <v>45705</v>
-      </c>
-      <c r="C377" t="inlineStr">
-        <is>
-          <t>Rahul</t>
-        </is>
-      </c>
-      <c r="D377" t="inlineStr">
-        <is>
-          <t>rahul71@gmail.com</t>
-        </is>
-      </c>
-      <c r="E377" t="n">
-        <v>9789375429</v>
-      </c>
-      <c r="F377" t="inlineStr">
-        <is>
-          <t>Lucknow</t>
-        </is>
-      </c>
-      <c r="G377" t="inlineStr">
-        <is>
-          <t>Up</t>
-        </is>
-      </c>
-      <c r="H377" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="I377" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="J377" t="n">
-        <v>4</v>
-      </c>
-      <c r="K377" t="n">
-        <v>9999</v>
-      </c>
-      <c r="L377" t="n">
-        <v>0</v>
-      </c>
-      <c r="M377" t="inlineStr">
-        <is>
-          <t>Card</t>
-        </is>
-      </c>
-      <c r="N377" t="inlineStr">
-        <is>
-          <t>Returned</t>
-        </is>
-      </c>
-      <c r="O377" s="2" t="n">
-        <v>45705</v>
-      </c>
-      <c r="P377" t="n">
-        <v>39996</v>
-      </c>
-      <c r="Q377" t="n">
-        <v>39996</v>
-      </c>
-      <c r="R377" t="n">
-        <v>7999.200000000001</v>
-      </c>
-      <c r="S377" t="inlineStr">
-        <is>
-          <t>February</t>
-        </is>
-      </c>
-      <c r="T377" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U377" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" t="inlineStr">
-        <is>
-          <t>ORD1609</t>
-        </is>
-      </c>
-      <c r="B378" t="inlineStr"/>
-      <c r="C378" t="inlineStr">
-        <is>
-          <t>Rahul</t>
-        </is>
-      </c>
-      <c r="D378" t="inlineStr">
-        <is>
-          <t>rahul99@gmail.com</t>
-        </is>
-      </c>
-      <c r="E378" t="n">
-        <v>9552649559</v>
-      </c>
-      <c r="F378" t="inlineStr">
-        <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="G378" t="inlineStr">
-        <is>
-          <t>Maharashtra</t>
-        </is>
-      </c>
-      <c r="H378" t="inlineStr">
-        <is>
-          <t>Bottle</t>
-        </is>
-      </c>
-      <c r="I378" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="J378" t="n">
-        <v>2</v>
-      </c>
-      <c r="K378" t="n">
-        <v>1499</v>
-      </c>
-      <c r="L378" t="n">
-        <v>0</v>
-      </c>
-      <c r="M378" t="inlineStr">
-        <is>
-          <t>Wallet</t>
-        </is>
-      </c>
-      <c r="N378" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="O378" t="inlineStr"/>
-      <c r="P378" t="n">
-        <v>2998</v>
-      </c>
-      <c r="Q378" t="n">
-        <v>2998</v>
-      </c>
-      <c r="R378" t="n">
-        <v>599.6</v>
-      </c>
-      <c r="S378" t="inlineStr"/>
-      <c r="T378" t="inlineStr"/>
-      <c r="U378" t="inlineStr"/>
-    </row>
-    <row r="379">
-      <c r="A379" t="inlineStr">
-        <is>
-          <t>ORD1610</t>
-        </is>
-      </c>
-      <c r="B379" s="2" t="n">
-        <v>45757</v>
-      </c>
-      <c r="C379" t="inlineStr">
-        <is>
-          <t>Rohit</t>
-        </is>
-      </c>
-      <c r="D379" t="inlineStr">
-        <is>
-          <t>rohit96@gmail.com</t>
-        </is>
-      </c>
-      <c r="E379" t="n">
-        <v>9700116928</v>
-      </c>
-      <c r="F379" t="inlineStr">
-        <is>
-          <t>Jaipur</t>
-        </is>
-      </c>
-      <c r="G379" t="inlineStr">
-        <is>
-          <t>Rajasthan</t>
-        </is>
-      </c>
-      <c r="H379" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="I379" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
-      <c r="J379" t="n">
-        <v>1</v>
-      </c>
-      <c r="K379" t="inlineStr"/>
-      <c r="L379" t="n">
-        <v>0</v>
-      </c>
-      <c r="M379" t="inlineStr">
-        <is>
-          <t>NetBanking</t>
-        </is>
-      </c>
-      <c r="N379" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
-      <c r="O379" s="2" t="n">
-        <v>45757</v>
-      </c>
-      <c r="P379" t="inlineStr"/>
-      <c r="Q379" t="inlineStr"/>
-      <c r="R379" t="inlineStr"/>
-      <c r="S379" t="inlineStr">
-        <is>
-          <t>April</t>
-        </is>
-      </c>
-      <c r="T379" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U379" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" t="inlineStr">
-        <is>
-          <t>ORD1611</t>
-        </is>
-      </c>
-      <c r="B380" s="2" t="n">
-        <v>45668</v>
-      </c>
-      <c r="C380" t="inlineStr">
-        <is>
-          <t>Neha</t>
-        </is>
-      </c>
-      <c r="D380" t="inlineStr">
-        <is>
-          <t>neha22@gmail.com</t>
-        </is>
-      </c>
-      <c r="E380" t="n">
-        <v>9580304152</v>
-      </c>
-      <c r="F380" t="inlineStr">
-        <is>
-          <t>Jaipur</t>
-        </is>
-      </c>
-      <c r="G380" t="inlineStr">
-        <is>
-          <t>Rajasthan</t>
-        </is>
-      </c>
-      <c r="H380" t="inlineStr">
-        <is>
-          <t>Chair</t>
-        </is>
-      </c>
-      <c r="I380" t="inlineStr">
-        <is>
-          <t>Furniture</t>
-        </is>
-      </c>
-      <c r="J380" t="n">
-        <v>3</v>
-      </c>
-      <c r="K380" t="n">
-        <v>999</v>
-      </c>
-      <c r="L380" t="n">
-        <v>0</v>
-      </c>
-      <c r="M380" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="N380" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="O380" s="2" t="n">
-        <v>45668</v>
-      </c>
-      <c r="P380" t="n">
-        <v>2997</v>
-      </c>
-      <c r="Q380" t="n">
-        <v>2997</v>
-      </c>
-      <c r="R380" t="n">
-        <v>599.4</v>
-      </c>
-      <c r="S380" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="T380" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U380" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" t="inlineStr">
-        <is>
-          <t>ORD1612</t>
-        </is>
-      </c>
-      <c r="B381" s="2" t="n">
-        <v>45719</v>
-      </c>
-      <c r="C381" t="inlineStr">
-        <is>
-          <t>Vikas</t>
-        </is>
-      </c>
-      <c r="D381" t="inlineStr">
-        <is>
-          <t>vikas46@gmail.com</t>
-        </is>
-      </c>
-      <c r="E381" t="n">
-        <v>9551158398</v>
-      </c>
-      <c r="F381" t="inlineStr">
-        <is>
-          <t>Jaipur</t>
-        </is>
-      </c>
-      <c r="G381" t="inlineStr">
-        <is>
-          <t>Rajasthan</t>
-        </is>
-      </c>
-      <c r="H381" t="inlineStr">
-        <is>
-          <t>Shoes</t>
-        </is>
-      </c>
-      <c r="I381" t="inlineStr">
-        <is>
-          <t>Fashion</t>
-        </is>
-      </c>
-      <c r="J381" t="n">
-        <v>3</v>
-      </c>
-      <c r="K381" t="n">
-        <v>999</v>
-      </c>
-      <c r="L381" t="n">
-        <v>5</v>
-      </c>
-      <c r="M381" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="N381" t="inlineStr">
-        <is>
-          <t>Cancelled</t>
-        </is>
-      </c>
-      <c r="O381" s="2" t="n">
-        <v>45903</v>
-      </c>
-      <c r="P381" t="n">
-        <v>2997</v>
-      </c>
-      <c r="Q381" t="n">
-        <v>2847.15</v>
-      </c>
-      <c r="R381" t="n">
-        <v>569.4300000000001</v>
-      </c>
-      <c r="S381" t="inlineStr">
-        <is>
-          <t>March</t>
-        </is>
-      </c>
-      <c r="T381" t="n">
-        <v>2025</v>
-      </c>
-      <c r="U381" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>